<commit_message>
Generate the PRISMA counts and the other counts the text quotes
A PRISMA sheet in the workbook holds the per-database search counts
and the screening and full-text exclusions; the split between the
database search and citation searching comes from Selected_articles'
Source column. The generator checks that counts never rise between
search stages, that the IEEE conference and journal counts add up,
and that databases + citation searching = the number of studies,
and warns about any study with no Source.

It also writes the domain and year shares, the top three countries'
counts and shares, the airborne, feedforward-network and Remote
Sensing counts, NDVI/NDWI/EVI use among satellite studies, each DEM
source's count, and the number of African countries absent from
the corpus. fig-prisma.tex now takes every count from numbers.tex.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/source/Reviewed_articles_only.xlsx
+++ b/figures/source/Reviewed_articles_only.xlsx
@@ -18,9 +18,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="task_long" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms_long" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="journals_long" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRISMA" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Studies'!$A$1:$Y$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'PRISMA'!$A$1:$C$41</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -20376,6 +20378,638 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Web of Science</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Scopus</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IEEE Xplore</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Google Scholar Labs</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>In 2015-2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Web of Science</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>In 2015-2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Scopus</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>In 2015-2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IEEE Xplore</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>In 2015-2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>In 2015-2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Google Scholar Labs</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Web of Science</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Scopus</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IEEE Xplore</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Google Scholar Labs</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Web of Science</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Scopus</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IEEE Xplore</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Google Scholar Labs</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Carried forward</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Web of Science</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Carried forward</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Scopus</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Carried forward</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IEEE Xplore</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Carried forward</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Carried forward</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Google Scholar Labs</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>IEEE Xplore by type</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Conference, returned</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IEEE Xplore by type</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Journal, returned</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>IEEE Xplore by type</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Conference, in 2015-2026</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IEEE Xplore by type</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Journal, in 2015-2026</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Duplicates removed</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>All databases</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Excluded at screening</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Excluded at screening</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Global scope</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Excluded at screening</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Excluded at screening</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Outside Africa</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Not retrieved</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Full text unavailable</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Excluded at full text</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Off-theme</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Excluded at full text</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Insufficient depth</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Excluded at full text</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>No EO data</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Excluded at full text</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Publication type</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Excluded at full text</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C41"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>